<commit_message>
Marcar atividade 25 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1629,7 +1629,7 @@
         <v>30</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J26" t="b">
         <v>0</v>
@@ -1721,13 +1721,17 @@
         <v>30</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-29 21:06</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2181,7 +2185,7 @@
         <v>30</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J38" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Marcar atividade 11 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -985,13 +985,17 @@
         <v>30</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-29 21:06</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1169,13 +1173,17 @@
         <v>60</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-29 21:06</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">

</xml_diff>

<commit_message>
Marcar atividade 9 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -893,13 +893,17 @@
         <v>30</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-29 21:06</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">

</xml_diff>

<commit_message>
Atalho PWA: Mairo Vergara concluído (Admin, ref. 2026-08-31)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -540,16 +540,16 @@
         <v>30</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>Marcado via atalho PWA (Mairo Vergara)</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>2026-09-29 18:07</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Atalho PWA: English Live concluído (Admin, ref. 2026-08-31)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -578,16 +578,16 @@
         <v>45</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>Marcado via atalho PWA (English Live)</v>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>2026-09-29 18:08</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Atalho PWA: Mairo Vergara concluído (Admin, ref. 2026-09-01)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -616,16 +616,16 @@
         <v>20</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>Marcado via atalho PWA (Mairo Vergara)</v>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>2026-09-29 18:11</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Reorganizar estudos de Admin (perfil atualizado)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -4033,7 +4033,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>849</v>
+        <v>1220</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>850</v>
+        <v>1221</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -4125,7 +4125,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>851</v>
+        <v>1222</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -4171,7 +4171,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>852</v>
+        <v>1223</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>853</v>
+        <v>1224</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -4263,7 +4263,7 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>854</v>
+        <v>1225</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -4309,7 +4309,7 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>855</v>
+        <v>1226</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -4355,7 +4355,7 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>856</v>
+        <v>1227</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>857</v>
+        <v>1228</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>858</v>
+        <v>1229</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -4493,7 +4493,7 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>859</v>
+        <v>1230</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -4539,7 +4539,7 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>860</v>
+        <v>1231</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -4585,7 +4585,7 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>861</v>
+        <v>1232</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -4631,7 +4631,7 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>862</v>
+        <v>1233</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -4677,7 +4677,7 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>863</v>
+        <v>1234</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>864</v>
+        <v>1235</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -4769,7 +4769,7 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>865</v>
+        <v>1236</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -4815,7 +4815,7 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>866</v>
+        <v>1237</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -4861,7 +4861,7 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>867</v>
+        <v>1238</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -4907,7 +4907,7 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>868</v>
+        <v>1239</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -4953,7 +4953,7 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>869</v>
+        <v>1240</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -4999,7 +4999,7 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>870</v>
+        <v>1241</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -5045,7 +5045,7 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>871</v>
+        <v>1242</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -5091,7 +5091,7 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>872</v>
+        <v>1243</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -5137,7 +5137,7 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>873</v>
+        <v>1244</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>874</v>
+        <v>1245</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -5229,7 +5229,7 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>875</v>
+        <v>1246</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>876</v>
+        <v>1247</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -5321,7 +5321,7 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>877</v>
+        <v>1248</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -5367,7 +5367,7 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>878</v>
+        <v>1249</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -5413,7 +5413,7 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>879</v>
+        <v>1250</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -5459,7 +5459,7 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>880</v>
+        <v>1251</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -5505,7 +5505,7 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>881</v>
+        <v>1252</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -5551,7 +5551,7 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>882</v>
+        <v>1253</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -5597,7 +5597,7 @@
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>883</v>
+        <v>1254</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -5643,7 +5643,7 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>884</v>
+        <v>1255</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>885</v>
+        <v>1256</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -5735,7 +5735,7 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>886</v>
+        <v>1257</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -5781,7 +5781,7 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>887</v>
+        <v>1258</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -5827,7 +5827,7 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>888</v>
+        <v>1259</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>889</v>
+        <v>1260</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -5919,7 +5919,7 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>890</v>
+        <v>1261</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -5965,7 +5965,7 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>891</v>
+        <v>1262</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -6011,7 +6011,7 @@
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>892</v>
+        <v>1263</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>893</v>
+        <v>1264</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>894</v>
+        <v>1265</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -6149,7 +6149,7 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>895</v>
+        <v>1266</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -6195,7 +6195,7 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>896</v>
+        <v>1267</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -6241,7 +6241,7 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>897</v>
+        <v>1268</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -6287,7 +6287,7 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>898</v>
+        <v>1269</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -6333,7 +6333,7 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>899</v>
+        <v>1270</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -6379,7 +6379,7 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>900</v>
+        <v>1271</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -6425,7 +6425,7 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>901</v>
+        <v>1272</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -6471,7 +6471,7 @@
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>902</v>
+        <v>1273</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -6517,7 +6517,7 @@
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>903</v>
+        <v>1274</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -6563,7 +6563,7 @@
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>904</v>
+        <v>1275</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -6609,7 +6609,7 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>905</v>
+        <v>1276</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>906</v>
+        <v>1277</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -6701,7 +6701,7 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>907</v>
+        <v>1278</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -6747,7 +6747,7 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>908</v>
+        <v>1279</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -6793,7 +6793,7 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>909</v>
+        <v>1280</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -6839,7 +6839,7 @@
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>910</v>
+        <v>1281</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -6885,7 +6885,7 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>911</v>
+        <v>1282</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -6931,7 +6931,7 @@
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>912</v>
+        <v>1283</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -6977,7 +6977,7 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>913</v>
+        <v>1284</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>914</v>
+        <v>1285</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -7069,7 +7069,7 @@
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>915</v>
+        <v>1286</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -7115,7 +7115,7 @@
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>916</v>
+        <v>1287</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -7161,7 +7161,7 @@
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>917</v>
+        <v>1288</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -7207,7 +7207,7 @@
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>918</v>
+        <v>1289</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -7253,7 +7253,7 @@
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>919</v>
+        <v>1290</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -7299,7 +7299,7 @@
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>920</v>
+        <v>1291</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -7345,7 +7345,7 @@
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>921</v>
+        <v>1292</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -7391,7 +7391,7 @@
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>922</v>
+        <v>1293</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -7437,7 +7437,7 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>923</v>
+        <v>1294</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -7483,7 +7483,7 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>924</v>
+        <v>1295</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -7529,7 +7529,7 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>925</v>
+        <v>1296</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -7575,7 +7575,7 @@
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>926</v>
+        <v>1297</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -7621,7 +7621,7 @@
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>927</v>
+        <v>1298</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -7667,7 +7667,7 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>928</v>
+        <v>1299</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -7713,7 +7713,7 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>929</v>
+        <v>1300</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -7759,7 +7759,7 @@
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>930</v>
+        <v>1301</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -7805,7 +7805,7 @@
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>931</v>
+        <v>1302</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -7851,7 +7851,7 @@
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>932</v>
+        <v>1303</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -7897,7 +7897,7 @@
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>933</v>
+        <v>1304</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -7943,7 +7943,7 @@
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>934</v>
+        <v>1305</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -7989,7 +7989,7 @@
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>935</v>
+        <v>1306</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -8035,7 +8035,7 @@
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>936</v>
+        <v>1307</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>937</v>
+        <v>1308</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -8127,7 +8127,7 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>938</v>
+        <v>1309</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -8173,7 +8173,7 @@
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>939</v>
+        <v>1310</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -8219,7 +8219,7 @@
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>940</v>
+        <v>1311</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -8265,7 +8265,7 @@
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>941</v>
+        <v>1312</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -8311,7 +8311,7 @@
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>942</v>
+        <v>1313</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -8357,7 +8357,7 @@
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>943</v>
+        <v>1314</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -8403,7 +8403,7 @@
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>944</v>
+        <v>1315</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -8449,7 +8449,7 @@
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>945</v>
+        <v>1316</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -8495,7 +8495,7 @@
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>946</v>
+        <v>1317</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -8541,7 +8541,7 @@
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>947</v>
+        <v>1318</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -8587,7 +8587,7 @@
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>948</v>
+        <v>1319</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -8633,7 +8633,7 @@
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>949</v>
+        <v>1320</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -8679,7 +8679,7 @@
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>950</v>
+        <v>1321</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -8725,7 +8725,7 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>951</v>
+        <v>1322</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -8771,7 +8771,7 @@
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>952</v>
+        <v>1323</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -8817,7 +8817,7 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>953</v>
+        <v>1324</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -8863,7 +8863,7 @@
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>954</v>
+        <v>1325</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -8909,7 +8909,7 @@
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>955</v>
+        <v>1326</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -8955,7 +8955,7 @@
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>956</v>
+        <v>1327</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -9001,7 +9001,7 @@
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>957</v>
+        <v>1328</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -9047,7 +9047,7 @@
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>958</v>
+        <v>1329</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -9093,7 +9093,7 @@
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>959</v>
+        <v>1330</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -9139,7 +9139,7 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>960</v>
+        <v>1331</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -9185,7 +9185,7 @@
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>961</v>
+        <v>1332</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -9231,7 +9231,7 @@
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>962</v>
+        <v>1333</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -9277,7 +9277,7 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>963</v>
+        <v>1334</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -9323,7 +9323,7 @@
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>964</v>
+        <v>1335</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -9369,7 +9369,7 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>965</v>
+        <v>1336</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -9415,7 +9415,7 @@
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>966</v>
+        <v>1337</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -9461,7 +9461,7 @@
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>967</v>
+        <v>1338</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -9507,7 +9507,7 @@
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>968</v>
+        <v>1339</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -9553,7 +9553,7 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>969</v>
+        <v>1340</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -9599,7 +9599,7 @@
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>970</v>
+        <v>1341</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -9645,7 +9645,7 @@
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>971</v>
+        <v>1342</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -9691,7 +9691,7 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>972</v>
+        <v>1343</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -9737,7 +9737,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>973</v>
+        <v>1344</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -9783,7 +9783,7 @@
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>974</v>
+        <v>1345</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -9829,7 +9829,7 @@
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>975</v>
+        <v>1346</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -9875,7 +9875,7 @@
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>976</v>
+        <v>1347</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -9921,7 +9921,7 @@
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>977</v>
+        <v>1348</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -9967,7 +9967,7 @@
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>978</v>
+        <v>1349</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -10013,7 +10013,7 @@
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>979</v>
+        <v>1350</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -10059,7 +10059,7 @@
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>980</v>
+        <v>1351</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -10105,7 +10105,7 @@
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>981</v>
+        <v>1352</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -10151,7 +10151,7 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>982</v>
+        <v>1353</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>983</v>
+        <v>1354</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
@@ -10243,7 +10243,7 @@
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>984</v>
+        <v>1355</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
@@ -10289,7 +10289,7 @@
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>985</v>
+        <v>1356</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -10335,7 +10335,7 @@
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>986</v>
+        <v>1357</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -10381,7 +10381,7 @@
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>987</v>
+        <v>1358</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
@@ -10427,7 +10427,7 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>988</v>
+        <v>1359</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -10473,7 +10473,7 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>989</v>
+        <v>1360</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -10519,7 +10519,7 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>990</v>
+        <v>1361</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -10565,7 +10565,7 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>991</v>
+        <v>1362</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -10611,7 +10611,7 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>992</v>
+        <v>1363</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -10657,7 +10657,7 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>993</v>
+        <v>1364</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -10703,7 +10703,7 @@
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>994</v>
+        <v>1365</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -10749,7 +10749,7 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>995</v>
+        <v>1366</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -10795,7 +10795,7 @@
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>996</v>
+        <v>1367</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -10841,7 +10841,7 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>997</v>
+        <v>1368</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -10887,7 +10887,7 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>998</v>
+        <v>1369</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -10933,7 +10933,7 @@
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>999</v>
+        <v>1370</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -10979,7 +10979,7 @@
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>1000</v>
+        <v>1371</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -11025,7 +11025,7 @@
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>1001</v>
+        <v>1372</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -11071,7 +11071,7 @@
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>1002</v>
+        <v>1373</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -11117,7 +11117,7 @@
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>1003</v>
+        <v>1374</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
@@ -11163,7 +11163,7 @@
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>1004</v>
+        <v>1375</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -11209,7 +11209,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>1005</v>
+        <v>1376</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -11255,7 +11255,7 @@
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>1006</v>
+        <v>1377</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -11301,7 +11301,7 @@
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>1007</v>
+        <v>1378</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
@@ -11347,7 +11347,7 @@
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>1008</v>
+        <v>1379</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
@@ -11393,7 +11393,7 @@
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>1009</v>
+        <v>1380</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>1010</v>
+        <v>1381</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
@@ -11485,7 +11485,7 @@
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>1011</v>
+        <v>1382</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
@@ -11531,7 +11531,7 @@
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>1012</v>
+        <v>1383</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
@@ -11577,7 +11577,7 @@
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>1013</v>
+        <v>1384</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
@@ -11623,7 +11623,7 @@
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>1014</v>
+        <v>1385</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
@@ -11669,7 +11669,7 @@
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>1015</v>
+        <v>1386</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
@@ -11715,7 +11715,7 @@
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>1016</v>
+        <v>1387</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
@@ -11761,7 +11761,7 @@
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>1017</v>
+        <v>1388</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
@@ -11807,7 +11807,7 @@
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>1018</v>
+        <v>1389</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
@@ -11853,7 +11853,7 @@
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>1019</v>
+        <v>1390</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
@@ -11899,7 +11899,7 @@
     </row>
     <row r="249">
       <c r="A249" t="n">
-        <v>1020</v>
+        <v>1391</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
@@ -11945,7 +11945,7 @@
     </row>
     <row r="250">
       <c r="A250" t="n">
-        <v>1021</v>
+        <v>1392</v>
       </c>
       <c r="B250" t="inlineStr">
         <is>
@@ -11991,7 +11991,7 @@
     </row>
     <row r="251">
       <c r="A251" t="n">
-        <v>1022</v>
+        <v>1393</v>
       </c>
       <c r="B251" t="inlineStr">
         <is>
@@ -12037,7 +12037,7 @@
     </row>
     <row r="252">
       <c r="A252" t="n">
-        <v>1023</v>
+        <v>1394</v>
       </c>
       <c r="B252" t="inlineStr">
         <is>
@@ -12083,7 +12083,7 @@
     </row>
     <row r="253">
       <c r="A253" t="n">
-        <v>1024</v>
+        <v>1395</v>
       </c>
       <c r="B253" t="inlineStr">
         <is>
@@ -12129,7 +12129,7 @@
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>1025</v>
+        <v>1396</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
@@ -12175,7 +12175,7 @@
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>1026</v>
+        <v>1397</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
@@ -12221,7 +12221,7 @@
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>1027</v>
+        <v>1398</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
@@ -12267,7 +12267,7 @@
     </row>
     <row r="257">
       <c r="A257" t="n">
-        <v>1028</v>
+        <v>1399</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
@@ -12313,7 +12313,7 @@
     </row>
     <row r="258">
       <c r="A258" t="n">
-        <v>1029</v>
+        <v>1400</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
@@ -12359,7 +12359,7 @@
     </row>
     <row r="259">
       <c r="A259" t="n">
-        <v>1030</v>
+        <v>1401</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
@@ -12405,7 +12405,7 @@
     </row>
     <row r="260">
       <c r="A260" t="n">
-        <v>1031</v>
+        <v>1402</v>
       </c>
       <c r="B260" t="inlineStr">
         <is>
@@ -12451,7 +12451,7 @@
     </row>
     <row r="261">
       <c r="A261" t="n">
-        <v>1032</v>
+        <v>1403</v>
       </c>
       <c r="B261" t="inlineStr">
         <is>
@@ -12497,7 +12497,7 @@
     </row>
     <row r="262">
       <c r="A262" t="n">
-        <v>1033</v>
+        <v>1404</v>
       </c>
       <c r="B262" t="inlineStr">
         <is>
@@ -12543,7 +12543,7 @@
     </row>
     <row r="263">
       <c r="A263" t="n">
-        <v>1034</v>
+        <v>1405</v>
       </c>
       <c r="B263" t="inlineStr">
         <is>
@@ -12589,7 +12589,7 @@
     </row>
     <row r="264">
       <c r="A264" t="n">
-        <v>1035</v>
+        <v>1406</v>
       </c>
       <c r="B264" t="inlineStr">
         <is>
@@ -12635,7 +12635,7 @@
     </row>
     <row r="265">
       <c r="A265" t="n">
-        <v>1036</v>
+        <v>1407</v>
       </c>
       <c r="B265" t="inlineStr">
         <is>
@@ -12681,7 +12681,7 @@
     </row>
     <row r="266">
       <c r="A266" t="n">
-        <v>1037</v>
+        <v>1408</v>
       </c>
       <c r="B266" t="inlineStr">
         <is>
@@ -12727,7 +12727,7 @@
     </row>
     <row r="267">
       <c r="A267" t="n">
-        <v>1038</v>
+        <v>1409</v>
       </c>
       <c r="B267" t="inlineStr">
         <is>
@@ -12773,7 +12773,7 @@
     </row>
     <row r="268">
       <c r="A268" t="n">
-        <v>1039</v>
+        <v>1410</v>
       </c>
       <c r="B268" t="inlineStr">
         <is>
@@ -12819,7 +12819,7 @@
     </row>
     <row r="269">
       <c r="A269" t="n">
-        <v>1040</v>
+        <v>1411</v>
       </c>
       <c r="B269" t="inlineStr">
         <is>
@@ -12865,7 +12865,7 @@
     </row>
     <row r="270">
       <c r="A270" t="n">
-        <v>1041</v>
+        <v>1412</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
@@ -12911,7 +12911,7 @@
     </row>
     <row r="271">
       <c r="A271" t="n">
-        <v>1042</v>
+        <v>1413</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
@@ -12957,7 +12957,7 @@
     </row>
     <row r="272">
       <c r="A272" t="n">
-        <v>1043</v>
+        <v>1414</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
@@ -13003,7 +13003,7 @@
     </row>
     <row r="273">
       <c r="A273" t="n">
-        <v>1044</v>
+        <v>1415</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
@@ -13049,7 +13049,7 @@
     </row>
     <row r="274">
       <c r="A274" t="n">
-        <v>1045</v>
+        <v>1416</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
@@ -13095,7 +13095,7 @@
     </row>
     <row r="275">
       <c r="A275" t="n">
-        <v>1046</v>
+        <v>1417</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
@@ -13141,7 +13141,7 @@
     </row>
     <row r="276">
       <c r="A276" t="n">
-        <v>1047</v>
+        <v>1418</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
@@ -13187,7 +13187,7 @@
     </row>
     <row r="277">
       <c r="A277" t="n">
-        <v>1048</v>
+        <v>1419</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
@@ -13233,7 +13233,7 @@
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>1049</v>
+        <v>1420</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
@@ -13279,7 +13279,7 @@
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>1050</v>
+        <v>1421</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
@@ -13325,7 +13325,7 @@
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>1051</v>
+        <v>1422</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
@@ -13371,7 +13371,7 @@
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>1052</v>
+        <v>1423</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
@@ -13417,7 +13417,7 @@
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>1053</v>
+        <v>1424</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
@@ -13463,7 +13463,7 @@
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>1054</v>
+        <v>1425</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
@@ -13509,7 +13509,7 @@
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>1055</v>
+        <v>1426</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
@@ -13555,7 +13555,7 @@
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>1056</v>
+        <v>1427</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
@@ -13601,7 +13601,7 @@
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>1057</v>
+        <v>1428</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
@@ -13647,7 +13647,7 @@
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>1058</v>
+        <v>1429</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
@@ -13693,7 +13693,7 @@
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>1059</v>
+        <v>1430</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
@@ -13739,7 +13739,7 @@
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>1060</v>
+        <v>1431</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
@@ -13785,7 +13785,7 @@
     </row>
     <row r="290">
       <c r="A290" t="n">
-        <v>1061</v>
+        <v>1432</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
@@ -13831,7 +13831,7 @@
     </row>
     <row r="291">
       <c r="A291" t="n">
-        <v>1062</v>
+        <v>1433</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
@@ -13877,7 +13877,7 @@
     </row>
     <row r="292">
       <c r="A292" t="n">
-        <v>1063</v>
+        <v>1434</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
@@ -13923,7 +13923,7 @@
     </row>
     <row r="293">
       <c r="A293" t="n">
-        <v>1064</v>
+        <v>1435</v>
       </c>
       <c r="B293" t="inlineStr">
         <is>
@@ -13969,7 +13969,7 @@
     </row>
     <row r="294">
       <c r="A294" t="n">
-        <v>1065</v>
+        <v>1436</v>
       </c>
       <c r="B294" t="inlineStr">
         <is>
@@ -14015,7 +14015,7 @@
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>1066</v>
+        <v>1437</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
@@ -14061,7 +14061,7 @@
     </row>
     <row r="296">
       <c r="A296" t="n">
-        <v>1067</v>
+        <v>1438</v>
       </c>
       <c r="B296" t="inlineStr">
         <is>
@@ -14107,7 +14107,7 @@
     </row>
     <row r="297">
       <c r="A297" t="n">
-        <v>1068</v>
+        <v>1439</v>
       </c>
       <c r="B297" t="inlineStr">
         <is>
@@ -14153,7 +14153,7 @@
     </row>
     <row r="298">
       <c r="A298" t="n">
-        <v>1069</v>
+        <v>1440</v>
       </c>
       <c r="B298" t="inlineStr">
         <is>
@@ -14199,7 +14199,7 @@
     </row>
     <row r="299">
       <c r="A299" t="n">
-        <v>1070</v>
+        <v>1441</v>
       </c>
       <c r="B299" t="inlineStr">
         <is>
@@ -14245,7 +14245,7 @@
     </row>
     <row r="300">
       <c r="A300" t="n">
-        <v>1071</v>
+        <v>1442</v>
       </c>
       <c r="B300" t="inlineStr">
         <is>
@@ -14291,7 +14291,7 @@
     </row>
     <row r="301">
       <c r="A301" t="n">
-        <v>1072</v>
+        <v>1443</v>
       </c>
       <c r="B301" t="inlineStr">
         <is>
@@ -14337,7 +14337,7 @@
     </row>
     <row r="302">
       <c r="A302" t="n">
-        <v>1073</v>
+        <v>1444</v>
       </c>
       <c r="B302" t="inlineStr">
         <is>
@@ -14383,7 +14383,7 @@
     </row>
     <row r="303">
       <c r="A303" t="n">
-        <v>1074</v>
+        <v>1445</v>
       </c>
       <c r="B303" t="inlineStr">
         <is>
@@ -14429,7 +14429,7 @@
     </row>
     <row r="304">
       <c r="A304" t="n">
-        <v>1075</v>
+        <v>1446</v>
       </c>
       <c r="B304" t="inlineStr">
         <is>
@@ -14475,7 +14475,7 @@
     </row>
     <row r="305">
       <c r="A305" t="n">
-        <v>1076</v>
+        <v>1447</v>
       </c>
       <c r="B305" t="inlineStr">
         <is>
@@ -14521,7 +14521,7 @@
     </row>
     <row r="306">
       <c r="A306" t="n">
-        <v>1077</v>
+        <v>1448</v>
       </c>
       <c r="B306" t="inlineStr">
         <is>
@@ -14567,7 +14567,7 @@
     </row>
     <row r="307">
       <c r="A307" t="n">
-        <v>1078</v>
+        <v>1449</v>
       </c>
       <c r="B307" t="inlineStr">
         <is>
@@ -14613,7 +14613,7 @@
     </row>
     <row r="308">
       <c r="A308" t="n">
-        <v>1079</v>
+        <v>1450</v>
       </c>
       <c r="B308" t="inlineStr">
         <is>
@@ -14659,7 +14659,7 @@
     </row>
     <row r="309">
       <c r="A309" t="n">
-        <v>1080</v>
+        <v>1451</v>
       </c>
       <c r="B309" t="inlineStr">
         <is>
@@ -14705,7 +14705,7 @@
     </row>
     <row r="310">
       <c r="A310" t="n">
-        <v>1081</v>
+        <v>1452</v>
       </c>
       <c r="B310" t="inlineStr">
         <is>
@@ -14751,7 +14751,7 @@
     </row>
     <row r="311">
       <c r="A311" t="n">
-        <v>1082</v>
+        <v>1453</v>
       </c>
       <c r="B311" t="inlineStr">
         <is>
@@ -14797,7 +14797,7 @@
     </row>
     <row r="312">
       <c r="A312" t="n">
-        <v>1083</v>
+        <v>1454</v>
       </c>
       <c r="B312" t="inlineStr">
         <is>
@@ -14843,7 +14843,7 @@
     </row>
     <row r="313">
       <c r="A313" t="n">
-        <v>1084</v>
+        <v>1455</v>
       </c>
       <c r="B313" t="inlineStr">
         <is>
@@ -14889,7 +14889,7 @@
     </row>
     <row r="314">
       <c r="A314" t="n">
-        <v>1085</v>
+        <v>1456</v>
       </c>
       <c r="B314" t="inlineStr">
         <is>
@@ -14935,7 +14935,7 @@
     </row>
     <row r="315">
       <c r="A315" t="n">
-        <v>1086</v>
+        <v>1457</v>
       </c>
       <c r="B315" t="inlineStr">
         <is>
@@ -14981,7 +14981,7 @@
     </row>
     <row r="316">
       <c r="A316" t="n">
-        <v>1087</v>
+        <v>1458</v>
       </c>
       <c r="B316" t="inlineStr">
         <is>
@@ -15027,7 +15027,7 @@
     </row>
     <row r="317">
       <c r="A317" t="n">
-        <v>1088</v>
+        <v>1459</v>
       </c>
       <c r="B317" t="inlineStr">
         <is>
@@ -15073,7 +15073,7 @@
     </row>
     <row r="318">
       <c r="A318" t="n">
-        <v>1089</v>
+        <v>1460</v>
       </c>
       <c r="B318" t="inlineStr">
         <is>
@@ -15119,7 +15119,7 @@
     </row>
     <row r="319">
       <c r="A319" t="n">
-        <v>1090</v>
+        <v>1461</v>
       </c>
       <c r="B319" t="inlineStr">
         <is>
@@ -15165,7 +15165,7 @@
     </row>
     <row r="320">
       <c r="A320" t="n">
-        <v>1091</v>
+        <v>1462</v>
       </c>
       <c r="B320" t="inlineStr">
         <is>
@@ -15211,7 +15211,7 @@
     </row>
     <row r="321">
       <c r="A321" t="n">
-        <v>1092</v>
+        <v>1463</v>
       </c>
       <c r="B321" t="inlineStr">
         <is>
@@ -15257,7 +15257,7 @@
     </row>
     <row r="322">
       <c r="A322" t="n">
-        <v>1093</v>
+        <v>1464</v>
       </c>
       <c r="B322" t="inlineStr">
         <is>
@@ -15303,7 +15303,7 @@
     </row>
     <row r="323">
       <c r="A323" t="n">
-        <v>1094</v>
+        <v>1465</v>
       </c>
       <c r="B323" t="inlineStr">
         <is>
@@ -15349,7 +15349,7 @@
     </row>
     <row r="324">
       <c r="A324" t="n">
-        <v>1095</v>
+        <v>1466</v>
       </c>
       <c r="B324" t="inlineStr">
         <is>
@@ -15395,7 +15395,7 @@
     </row>
     <row r="325">
       <c r="A325" t="n">
-        <v>1096</v>
+        <v>1467</v>
       </c>
       <c r="B325" t="inlineStr">
         <is>
@@ -15441,7 +15441,7 @@
     </row>
     <row r="326">
       <c r="A326" t="n">
-        <v>1097</v>
+        <v>1468</v>
       </c>
       <c r="B326" t="inlineStr">
         <is>
@@ -15487,7 +15487,7 @@
     </row>
     <row r="327">
       <c r="A327" t="n">
-        <v>1098</v>
+        <v>1469</v>
       </c>
       <c r="B327" t="inlineStr">
         <is>
@@ -15533,7 +15533,7 @@
     </row>
     <row r="328">
       <c r="A328" t="n">
-        <v>1099</v>
+        <v>1470</v>
       </c>
       <c r="B328" t="inlineStr">
         <is>
@@ -15579,7 +15579,7 @@
     </row>
     <row r="329">
       <c r="A329" t="n">
-        <v>1100</v>
+        <v>1471</v>
       </c>
       <c r="B329" t="inlineStr">
         <is>
@@ -15625,7 +15625,7 @@
     </row>
     <row r="330">
       <c r="A330" t="n">
-        <v>1101</v>
+        <v>1472</v>
       </c>
       <c r="B330" t="inlineStr">
         <is>
@@ -15671,7 +15671,7 @@
     </row>
     <row r="331">
       <c r="A331" t="n">
-        <v>1102</v>
+        <v>1473</v>
       </c>
       <c r="B331" t="inlineStr">
         <is>
@@ -15717,7 +15717,7 @@
     </row>
     <row r="332">
       <c r="A332" t="n">
-        <v>1103</v>
+        <v>1474</v>
       </c>
       <c r="B332" t="inlineStr">
         <is>
@@ -15763,7 +15763,7 @@
     </row>
     <row r="333">
       <c r="A333" t="n">
-        <v>1104</v>
+        <v>1475</v>
       </c>
       <c r="B333" t="inlineStr">
         <is>
@@ -15809,7 +15809,7 @@
     </row>
     <row r="334">
       <c r="A334" t="n">
-        <v>1105</v>
+        <v>1476</v>
       </c>
       <c r="B334" t="inlineStr">
         <is>
@@ -15855,7 +15855,7 @@
     </row>
     <row r="335">
       <c r="A335" t="n">
-        <v>1106</v>
+        <v>1477</v>
       </c>
       <c r="B335" t="inlineStr">
         <is>
@@ -15901,7 +15901,7 @@
     </row>
     <row r="336">
       <c r="A336" t="n">
-        <v>1107</v>
+        <v>1478</v>
       </c>
       <c r="B336" t="inlineStr">
         <is>
@@ -15947,7 +15947,7 @@
     </row>
     <row r="337">
       <c r="A337" t="n">
-        <v>1108</v>
+        <v>1479</v>
       </c>
       <c r="B337" t="inlineStr">
         <is>
@@ -15993,7 +15993,7 @@
     </row>
     <row r="338">
       <c r="A338" t="n">
-        <v>1109</v>
+        <v>1480</v>
       </c>
       <c r="B338" t="inlineStr">
         <is>
@@ -16039,7 +16039,7 @@
     </row>
     <row r="339">
       <c r="A339" t="n">
-        <v>1110</v>
+        <v>1481</v>
       </c>
       <c r="B339" t="inlineStr">
         <is>
@@ -16085,7 +16085,7 @@
     </row>
     <row r="340">
       <c r="A340" t="n">
-        <v>1111</v>
+        <v>1482</v>
       </c>
       <c r="B340" t="inlineStr">
         <is>
@@ -16131,7 +16131,7 @@
     </row>
     <row r="341">
       <c r="A341" t="n">
-        <v>1112</v>
+        <v>1483</v>
       </c>
       <c r="B341" t="inlineStr">
         <is>
@@ -16177,7 +16177,7 @@
     </row>
     <row r="342">
       <c r="A342" t="n">
-        <v>1113</v>
+        <v>1484</v>
       </c>
       <c r="B342" t="inlineStr">
         <is>
@@ -16223,7 +16223,7 @@
     </row>
     <row r="343">
       <c r="A343" t="n">
-        <v>1114</v>
+        <v>1485</v>
       </c>
       <c r="B343" t="inlineStr">
         <is>
@@ -16269,7 +16269,7 @@
     </row>
     <row r="344">
       <c r="A344" t="n">
-        <v>1115</v>
+        <v>1486</v>
       </c>
       <c r="B344" t="inlineStr">
         <is>
@@ -16315,7 +16315,7 @@
     </row>
     <row r="345">
       <c r="A345" t="n">
-        <v>1116</v>
+        <v>1487</v>
       </c>
       <c r="B345" t="inlineStr">
         <is>
@@ -16361,7 +16361,7 @@
     </row>
     <row r="346">
       <c r="A346" t="n">
-        <v>1117</v>
+        <v>1488</v>
       </c>
       <c r="B346" t="inlineStr">
         <is>
@@ -16407,7 +16407,7 @@
     </row>
     <row r="347">
       <c r="A347" t="n">
-        <v>1118</v>
+        <v>1489</v>
       </c>
       <c r="B347" t="inlineStr">
         <is>
@@ -16453,7 +16453,7 @@
     </row>
     <row r="348">
       <c r="A348" t="n">
-        <v>1119</v>
+        <v>1490</v>
       </c>
       <c r="B348" t="inlineStr">
         <is>
@@ -16499,7 +16499,7 @@
     </row>
     <row r="349">
       <c r="A349" t="n">
-        <v>1120</v>
+        <v>1491</v>
       </c>
       <c r="B349" t="inlineStr">
         <is>
@@ -16545,7 +16545,7 @@
     </row>
     <row r="350">
       <c r="A350" t="n">
-        <v>1121</v>
+        <v>1492</v>
       </c>
       <c r="B350" t="inlineStr">
         <is>
@@ -16591,7 +16591,7 @@
     </row>
     <row r="351">
       <c r="A351" t="n">
-        <v>1122</v>
+        <v>1493</v>
       </c>
       <c r="B351" t="inlineStr">
         <is>
@@ -16637,7 +16637,7 @@
     </row>
     <row r="352">
       <c r="A352" t="n">
-        <v>1123</v>
+        <v>1494</v>
       </c>
       <c r="B352" t="inlineStr">
         <is>
@@ -16683,7 +16683,7 @@
     </row>
     <row r="353">
       <c r="A353" t="n">
-        <v>1124</v>
+        <v>1495</v>
       </c>
       <c r="B353" t="inlineStr">
         <is>
@@ -16729,7 +16729,7 @@
     </row>
     <row r="354">
       <c r="A354" t="n">
-        <v>1125</v>
+        <v>1496</v>
       </c>
       <c r="B354" t="inlineStr">
         <is>
@@ -16775,7 +16775,7 @@
     </row>
     <row r="355">
       <c r="A355" t="n">
-        <v>1126</v>
+        <v>1497</v>
       </c>
       <c r="B355" t="inlineStr">
         <is>
@@ -16821,7 +16821,7 @@
     </row>
     <row r="356">
       <c r="A356" t="n">
-        <v>1127</v>
+        <v>1498</v>
       </c>
       <c r="B356" t="inlineStr">
         <is>
@@ -16867,7 +16867,7 @@
     </row>
     <row r="357">
       <c r="A357" t="n">
-        <v>1128</v>
+        <v>1499</v>
       </c>
       <c r="B357" t="inlineStr">
         <is>
@@ -16913,7 +16913,7 @@
     </row>
     <row r="358">
       <c r="A358" t="n">
-        <v>1129</v>
+        <v>1500</v>
       </c>
       <c r="B358" t="inlineStr">
         <is>
@@ -16959,7 +16959,7 @@
     </row>
     <row r="359">
       <c r="A359" t="n">
-        <v>1130</v>
+        <v>1501</v>
       </c>
       <c r="B359" t="inlineStr">
         <is>
@@ -17005,7 +17005,7 @@
     </row>
     <row r="360">
       <c r="A360" t="n">
-        <v>1131</v>
+        <v>1502</v>
       </c>
       <c r="B360" t="inlineStr">
         <is>
@@ -17051,7 +17051,7 @@
     </row>
     <row r="361">
       <c r="A361" t="n">
-        <v>1132</v>
+        <v>1503</v>
       </c>
       <c r="B361" t="inlineStr">
         <is>
@@ -17097,7 +17097,7 @@
     </row>
     <row r="362">
       <c r="A362" t="n">
-        <v>1133</v>
+        <v>1504</v>
       </c>
       <c r="B362" t="inlineStr">
         <is>
@@ -17143,7 +17143,7 @@
     </row>
     <row r="363">
       <c r="A363" t="n">
-        <v>1134</v>
+        <v>1505</v>
       </c>
       <c r="B363" t="inlineStr">
         <is>
@@ -17189,7 +17189,7 @@
     </row>
     <row r="364">
       <c r="A364" t="n">
-        <v>1135</v>
+        <v>1506</v>
       </c>
       <c r="B364" t="inlineStr">
         <is>
@@ -17235,7 +17235,7 @@
     </row>
     <row r="365">
       <c r="A365" t="n">
-        <v>1136</v>
+        <v>1507</v>
       </c>
       <c r="B365" t="inlineStr">
         <is>
@@ -17281,7 +17281,7 @@
     </row>
     <row r="366">
       <c r="A366" t="n">
-        <v>1137</v>
+        <v>1508</v>
       </c>
       <c r="B366" t="inlineStr">
         <is>
@@ -17327,7 +17327,7 @@
     </row>
     <row r="367">
       <c r="A367" t="n">
-        <v>1138</v>
+        <v>1509</v>
       </c>
       <c r="B367" t="inlineStr">
         <is>
@@ -17373,7 +17373,7 @@
     </row>
     <row r="368">
       <c r="A368" t="n">
-        <v>1139</v>
+        <v>1510</v>
       </c>
       <c r="B368" t="inlineStr">
         <is>
@@ -17419,7 +17419,7 @@
     </row>
     <row r="369">
       <c r="A369" t="n">
-        <v>1140</v>
+        <v>1511</v>
       </c>
       <c r="B369" t="inlineStr">
         <is>
@@ -17465,7 +17465,7 @@
     </row>
     <row r="370">
       <c r="A370" t="n">
-        <v>1141</v>
+        <v>1512</v>
       </c>
       <c r="B370" t="inlineStr">
         <is>
@@ -17511,7 +17511,7 @@
     </row>
     <row r="371">
       <c r="A371" t="n">
-        <v>1142</v>
+        <v>1513</v>
       </c>
       <c r="B371" t="inlineStr">
         <is>
@@ -17557,7 +17557,7 @@
     </row>
     <row r="372">
       <c r="A372" t="n">
-        <v>1143</v>
+        <v>1514</v>
       </c>
       <c r="B372" t="inlineStr">
         <is>
@@ -17603,7 +17603,7 @@
     </row>
     <row r="373">
       <c r="A373" t="n">
-        <v>1144</v>
+        <v>1515</v>
       </c>
       <c r="B373" t="inlineStr">
         <is>
@@ -17649,7 +17649,7 @@
     </row>
     <row r="374">
       <c r="A374" t="n">
-        <v>1145</v>
+        <v>1516</v>
       </c>
       <c r="B374" t="inlineStr">
         <is>
@@ -17695,7 +17695,7 @@
     </row>
     <row r="375">
       <c r="A375" t="n">
-        <v>1146</v>
+        <v>1517</v>
       </c>
       <c r="B375" t="inlineStr">
         <is>
@@ -17741,7 +17741,7 @@
     </row>
     <row r="376">
       <c r="A376" t="n">
-        <v>1147</v>
+        <v>1518</v>
       </c>
       <c r="B376" t="inlineStr">
         <is>
@@ -17787,7 +17787,7 @@
     </row>
     <row r="377">
       <c r="A377" t="n">
-        <v>1148</v>
+        <v>1519</v>
       </c>
       <c r="B377" t="inlineStr">
         <is>
@@ -17833,7 +17833,7 @@
     </row>
     <row r="378">
       <c r="A378" t="n">
-        <v>1149</v>
+        <v>1520</v>
       </c>
       <c r="B378" t="inlineStr">
         <is>
@@ -17879,7 +17879,7 @@
     </row>
     <row r="379">
       <c r="A379" t="n">
-        <v>1150</v>
+        <v>1521</v>
       </c>
       <c r="B379" t="inlineStr">
         <is>
@@ -17925,7 +17925,7 @@
     </row>
     <row r="380">
       <c r="A380" t="n">
-        <v>1151</v>
+        <v>1522</v>
       </c>
       <c r="B380" t="inlineStr">
         <is>
@@ -17971,7 +17971,7 @@
     </row>
     <row r="381">
       <c r="A381" t="n">
-        <v>1152</v>
+        <v>1523</v>
       </c>
       <c r="B381" t="inlineStr">
         <is>
@@ -18017,7 +18017,7 @@
     </row>
     <row r="382">
       <c r="A382" t="n">
-        <v>1153</v>
+        <v>1524</v>
       </c>
       <c r="B382" t="inlineStr">
         <is>
@@ -18063,7 +18063,7 @@
     </row>
     <row r="383">
       <c r="A383" t="n">
-        <v>1154</v>
+        <v>1525</v>
       </c>
       <c r="B383" t="inlineStr">
         <is>
@@ -18109,7 +18109,7 @@
     </row>
     <row r="384">
       <c r="A384" t="n">
-        <v>1155</v>
+        <v>1526</v>
       </c>
       <c r="B384" t="inlineStr">
         <is>
@@ -18155,7 +18155,7 @@
     </row>
     <row r="385">
       <c r="A385" t="n">
-        <v>1156</v>
+        <v>1527</v>
       </c>
       <c r="B385" t="inlineStr">
         <is>
@@ -18201,7 +18201,7 @@
     </row>
     <row r="386">
       <c r="A386" t="n">
-        <v>1157</v>
+        <v>1528</v>
       </c>
       <c r="B386" t="inlineStr">
         <is>
@@ -18247,7 +18247,7 @@
     </row>
     <row r="387">
       <c r="A387" t="n">
-        <v>1158</v>
+        <v>1529</v>
       </c>
       <c r="B387" t="inlineStr">
         <is>
@@ -18293,7 +18293,7 @@
     </row>
     <row r="388">
       <c r="A388" t="n">
-        <v>1159</v>
+        <v>1530</v>
       </c>
       <c r="B388" t="inlineStr">
         <is>
@@ -18339,7 +18339,7 @@
     </row>
     <row r="389">
       <c r="A389" t="n">
-        <v>1160</v>
+        <v>1531</v>
       </c>
       <c r="B389" t="inlineStr">
         <is>
@@ -18385,7 +18385,7 @@
     </row>
     <row r="390">
       <c r="A390" t="n">
-        <v>1161</v>
+        <v>1532</v>
       </c>
       <c r="B390" t="inlineStr">
         <is>
@@ -18431,7 +18431,7 @@
     </row>
     <row r="391">
       <c r="A391" t="n">
-        <v>1162</v>
+        <v>1533</v>
       </c>
       <c r="B391" t="inlineStr">
         <is>
@@ -18477,7 +18477,7 @@
     </row>
     <row r="392">
       <c r="A392" t="n">
-        <v>1163</v>
+        <v>1534</v>
       </c>
       <c r="B392" t="inlineStr">
         <is>
@@ -18523,7 +18523,7 @@
     </row>
     <row r="393">
       <c r="A393" t="n">
-        <v>1164</v>
+        <v>1535</v>
       </c>
       <c r="B393" t="inlineStr">
         <is>
@@ -18569,7 +18569,7 @@
     </row>
     <row r="394">
       <c r="A394" t="n">
-        <v>1165</v>
+        <v>1536</v>
       </c>
       <c r="B394" t="inlineStr">
         <is>
@@ -18615,7 +18615,7 @@
     </row>
     <row r="395">
       <c r="A395" t="n">
-        <v>1166</v>
+        <v>1537</v>
       </c>
       <c r="B395" t="inlineStr">
         <is>
@@ -18661,7 +18661,7 @@
     </row>
     <row r="396">
       <c r="A396" t="n">
-        <v>1167</v>
+        <v>1538</v>
       </c>
       <c r="B396" t="inlineStr">
         <is>
@@ -18707,7 +18707,7 @@
     </row>
     <row r="397">
       <c r="A397" t="n">
-        <v>1168</v>
+        <v>1539</v>
       </c>
       <c r="B397" t="inlineStr">
         <is>
@@ -18753,7 +18753,7 @@
     </row>
     <row r="398">
       <c r="A398" t="n">
-        <v>1169</v>
+        <v>1540</v>
       </c>
       <c r="B398" t="inlineStr">
         <is>
@@ -18799,7 +18799,7 @@
     </row>
     <row r="399">
       <c r="A399" t="n">
-        <v>1170</v>
+        <v>1541</v>
       </c>
       <c r="B399" t="inlineStr">
         <is>
@@ -18845,7 +18845,7 @@
     </row>
     <row r="400">
       <c r="A400" t="n">
-        <v>1171</v>
+        <v>1542</v>
       </c>
       <c r="B400" t="inlineStr">
         <is>
@@ -18891,7 +18891,7 @@
     </row>
     <row r="401">
       <c r="A401" t="n">
-        <v>1172</v>
+        <v>1543</v>
       </c>
       <c r="B401" t="inlineStr">
         <is>
@@ -18937,7 +18937,7 @@
     </row>
     <row r="402">
       <c r="A402" t="n">
-        <v>1173</v>
+        <v>1544</v>
       </c>
       <c r="B402" t="inlineStr">
         <is>
@@ -18983,7 +18983,7 @@
     </row>
     <row r="403">
       <c r="A403" t="n">
-        <v>1174</v>
+        <v>1545</v>
       </c>
       <c r="B403" t="inlineStr">
         <is>
@@ -19029,7 +19029,7 @@
     </row>
     <row r="404">
       <c r="A404" t="n">
-        <v>1175</v>
+        <v>1546</v>
       </c>
       <c r="B404" t="inlineStr">
         <is>
@@ -19075,7 +19075,7 @@
     </row>
     <row r="405">
       <c r="A405" t="n">
-        <v>1176</v>
+        <v>1547</v>
       </c>
       <c r="B405" t="inlineStr">
         <is>
@@ -19121,7 +19121,7 @@
     </row>
     <row r="406">
       <c r="A406" t="n">
-        <v>1177</v>
+        <v>1548</v>
       </c>
       <c r="B406" t="inlineStr">
         <is>
@@ -19167,7 +19167,7 @@
     </row>
     <row r="407">
       <c r="A407" t="n">
-        <v>1178</v>
+        <v>1549</v>
       </c>
       <c r="B407" t="inlineStr">
         <is>
@@ -19213,7 +19213,7 @@
     </row>
     <row r="408">
       <c r="A408" t="n">
-        <v>1179</v>
+        <v>1550</v>
       </c>
       <c r="B408" t="inlineStr">
         <is>
@@ -19259,7 +19259,7 @@
     </row>
     <row r="409">
       <c r="A409" t="n">
-        <v>1180</v>
+        <v>1551</v>
       </c>
       <c r="B409" t="inlineStr">
         <is>
@@ -19305,7 +19305,7 @@
     </row>
     <row r="410">
       <c r="A410" t="n">
-        <v>1181</v>
+        <v>1552</v>
       </c>
       <c r="B410" t="inlineStr">
         <is>
@@ -19351,7 +19351,7 @@
     </row>
     <row r="411">
       <c r="A411" t="n">
-        <v>1182</v>
+        <v>1553</v>
       </c>
       <c r="B411" t="inlineStr">
         <is>
@@ -19397,7 +19397,7 @@
     </row>
     <row r="412">
       <c r="A412" t="n">
-        <v>1183</v>
+        <v>1554</v>
       </c>
       <c r="B412" t="inlineStr">
         <is>
@@ -19443,7 +19443,7 @@
     </row>
     <row r="413">
       <c r="A413" t="n">
-        <v>1184</v>
+        <v>1555</v>
       </c>
       <c r="B413" t="inlineStr">
         <is>
@@ -19489,7 +19489,7 @@
     </row>
     <row r="414">
       <c r="A414" t="n">
-        <v>1185</v>
+        <v>1556</v>
       </c>
       <c r="B414" t="inlineStr">
         <is>
@@ -19535,7 +19535,7 @@
     </row>
     <row r="415">
       <c r="A415" t="n">
-        <v>1186</v>
+        <v>1557</v>
       </c>
       <c r="B415" t="inlineStr">
         <is>
@@ -19581,7 +19581,7 @@
     </row>
     <row r="416">
       <c r="A416" t="n">
-        <v>1187</v>
+        <v>1558</v>
       </c>
       <c r="B416" t="inlineStr">
         <is>
@@ -19627,7 +19627,7 @@
     </row>
     <row r="417">
       <c r="A417" t="n">
-        <v>1188</v>
+        <v>1559</v>
       </c>
       <c r="B417" t="inlineStr">
         <is>
@@ -19673,7 +19673,7 @@
     </row>
     <row r="418">
       <c r="A418" t="n">
-        <v>1189</v>
+        <v>1560</v>
       </c>
       <c r="B418" t="inlineStr">
         <is>
@@ -19719,7 +19719,7 @@
     </row>
     <row r="419">
       <c r="A419" t="n">
-        <v>1190</v>
+        <v>1561</v>
       </c>
       <c r="B419" t="inlineStr">
         <is>
@@ -19765,7 +19765,7 @@
     </row>
     <row r="420">
       <c r="A420" t="n">
-        <v>1191</v>
+        <v>1562</v>
       </c>
       <c r="B420" t="inlineStr">
         <is>
@@ -19811,7 +19811,7 @@
     </row>
     <row r="421">
       <c r="A421" t="n">
-        <v>1192</v>
+        <v>1563</v>
       </c>
       <c r="B421" t="inlineStr">
         <is>
@@ -19857,7 +19857,7 @@
     </row>
     <row r="422">
       <c r="A422" t="n">
-        <v>1193</v>
+        <v>1564</v>
       </c>
       <c r="B422" t="inlineStr">
         <is>
@@ -19903,7 +19903,7 @@
     </row>
     <row r="423">
       <c r="A423" t="n">
-        <v>1194</v>
+        <v>1565</v>
       </c>
       <c r="B423" t="inlineStr">
         <is>
@@ -19949,7 +19949,7 @@
     </row>
     <row r="424">
       <c r="A424" t="n">
-        <v>1195</v>
+        <v>1566</v>
       </c>
       <c r="B424" t="inlineStr">
         <is>
@@ -19995,7 +19995,7 @@
     </row>
     <row r="425">
       <c r="A425" t="n">
-        <v>1196</v>
+        <v>1567</v>
       </c>
       <c r="B425" t="inlineStr">
         <is>
@@ -20041,7 +20041,7 @@
     </row>
     <row r="426">
       <c r="A426" t="n">
-        <v>1197</v>
+        <v>1568</v>
       </c>
       <c r="B426" t="inlineStr">
         <is>
@@ -20087,7 +20087,7 @@
     </row>
     <row r="427">
       <c r="A427" t="n">
-        <v>1198</v>
+        <v>1569</v>
       </c>
       <c r="B427" t="inlineStr">
         <is>
@@ -20133,7 +20133,7 @@
     </row>
     <row r="428">
       <c r="A428" t="n">
-        <v>1199</v>
+        <v>1570</v>
       </c>
       <c r="B428" t="inlineStr">
         <is>
@@ -20179,7 +20179,7 @@
     </row>
     <row r="429">
       <c r="A429" t="n">
-        <v>1200</v>
+        <v>1571</v>
       </c>
       <c r="B429" t="inlineStr">
         <is>
@@ -20225,7 +20225,7 @@
     </row>
     <row r="430">
       <c r="A430" t="n">
-        <v>1201</v>
+        <v>1572</v>
       </c>
       <c r="B430" t="inlineStr">
         <is>
@@ -20271,7 +20271,7 @@
     </row>
     <row r="431">
       <c r="A431" t="n">
-        <v>1202</v>
+        <v>1573</v>
       </c>
       <c r="B431" t="inlineStr">
         <is>
@@ -20317,7 +20317,7 @@
     </row>
     <row r="432">
       <c r="A432" t="n">
-        <v>1203</v>
+        <v>1574</v>
       </c>
       <c r="B432" t="inlineStr">
         <is>
@@ -20363,7 +20363,7 @@
     </row>
     <row r="433">
       <c r="A433" t="n">
-        <v>1204</v>
+        <v>1575</v>
       </c>
       <c r="B433" t="inlineStr">
         <is>
@@ -20409,7 +20409,7 @@
     </row>
     <row r="434">
       <c r="A434" t="n">
-        <v>1205</v>
+        <v>1576</v>
       </c>
       <c r="B434" t="inlineStr">
         <is>
@@ -20455,7 +20455,7 @@
     </row>
     <row r="435">
       <c r="A435" t="n">
-        <v>1206</v>
+        <v>1577</v>
       </c>
       <c r="B435" t="inlineStr">
         <is>
@@ -20501,7 +20501,7 @@
     </row>
     <row r="436">
       <c r="A436" t="n">
-        <v>1207</v>
+        <v>1578</v>
       </c>
       <c r="B436" t="inlineStr">
         <is>
@@ -20547,7 +20547,7 @@
     </row>
     <row r="437">
       <c r="A437" t="n">
-        <v>1208</v>
+        <v>1579</v>
       </c>
       <c r="B437" t="inlineStr">
         <is>
@@ -20593,7 +20593,7 @@
     </row>
     <row r="438">
       <c r="A438" t="n">
-        <v>1209</v>
+        <v>1580</v>
       </c>
       <c r="B438" t="inlineStr">
         <is>
@@ -20639,7 +20639,7 @@
     </row>
     <row r="439">
       <c r="A439" t="n">
-        <v>1210</v>
+        <v>1581</v>
       </c>
       <c r="B439" t="inlineStr">
         <is>
@@ -20685,7 +20685,7 @@
     </row>
     <row r="440">
       <c r="A440" t="n">
-        <v>1211</v>
+        <v>1582</v>
       </c>
       <c r="B440" t="inlineStr">
         <is>
@@ -20731,7 +20731,7 @@
     </row>
     <row r="441">
       <c r="A441" t="n">
-        <v>1212</v>
+        <v>1583</v>
       </c>
       <c r="B441" t="inlineStr">
         <is>
@@ -20777,7 +20777,7 @@
     </row>
     <row r="442">
       <c r="A442" t="n">
-        <v>1213</v>
+        <v>1584</v>
       </c>
       <c r="B442" t="inlineStr">
         <is>
@@ -20823,7 +20823,7 @@
     </row>
     <row r="443">
       <c r="A443" t="n">
-        <v>1214</v>
+        <v>1585</v>
       </c>
       <c r="B443" t="inlineStr">
         <is>
@@ -20869,7 +20869,7 @@
     </row>
     <row r="444">
       <c r="A444" t="n">
-        <v>1215</v>
+        <v>1586</v>
       </c>
       <c r="B444" t="inlineStr">
         <is>
@@ -20915,7 +20915,7 @@
     </row>
     <row r="445">
       <c r="A445" t="n">
-        <v>1216</v>
+        <v>1587</v>
       </c>
       <c r="B445" t="inlineStr">
         <is>
@@ -20961,7 +20961,7 @@
     </row>
     <row r="446">
       <c r="A446" t="n">
-        <v>1217</v>
+        <v>1588</v>
       </c>
       <c r="B446" t="inlineStr">
         <is>
@@ -21007,7 +21007,7 @@
     </row>
     <row r="447">
       <c r="A447" t="n">
-        <v>1218</v>
+        <v>1589</v>
       </c>
       <c r="B447" t="inlineStr">
         <is>
@@ -21053,7 +21053,7 @@
     </row>
     <row r="448">
       <c r="A448" t="n">
-        <v>1219</v>
+        <v>1590</v>
       </c>
       <c r="B448" t="inlineStr">
         <is>

</xml_diff>